<commit_message>
allowing custom probabilities for surveillance, along with a default value
</commit_message>
<xml_diff>
--- a/scenarios/v06/new_actions_1.xlsx
+++ b/scenarios/v06/new_actions_1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thaophuongl\Documents\HASTE_CODE\OutbreakSimulator\scenarios\v06\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\UNIMELB\outbreaksimulator\scenarios\v06\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FBAF289-9244-4ABE-8F65-65178A66271A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55B86FE0-9EB4-4F9E-AB0F-29E43CA38309}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{01539856-3AD6-4856-AAFB-F25B45651A69}"/>
+    <workbookView xWindow="33060" yWindow="285" windowWidth="21315" windowHeight="15075" activeTab="2" xr2:uid="{01539856-3AD6-4856-AAFB-F25B45651A69}"/>
   </bookViews>
   <sheets>
     <sheet name="jobs" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="54">
   <si>
     <t>ID</t>
   </si>
@@ -193,9 +193,6 @@
     </r>
   </si>
   <si>
-    <t>PopSurveillance</t>
-  </si>
-  <si>
     <t>EnhancedPassive</t>
   </si>
   <si>
@@ -208,7 +205,22 @@
     <t>(anything)</t>
   </si>
   <si>
-    <t xml:space="preserve">Used for PopSurveillance, identifier </t>
+    <t>missing detection probability - checking</t>
+  </si>
+  <si>
+    <t>zone_factor</t>
+  </si>
+  <si>
+    <t>PopulationSurveillance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Used for PopulationSurveillance as an identifier  for the zone </t>
+  </si>
+  <si>
+    <t>[a number]</t>
+  </si>
+  <si>
+    <t>optional: can be used for surveillance zones to adjust their success. Default values are "2" for enhancedpassive (twice as likely to have a self-report) and "0.9" for populationsurveillance (related to successful detection of HPAI in dead birds in a pooled PCR)</t>
   </si>
 </sst>
 </file>
@@ -250,12 +262,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -592,7 +603,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EC4FC7D-172B-4FB5-8C5B-14F92FDF678B}">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="17" customWidth="1"/>
@@ -802,7 +813,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>101</v>
       </c>
@@ -819,7 +830,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>500</v>
       </c>
@@ -834,6 +845,23 @@
       </c>
       <c r="E18">
         <v>0.2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>401</v>
+      </c>
+      <c r="B19" s="1">
+        <v>46036</v>
+      </c>
+      <c r="C19" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" t="s">
+        <v>38</v>
+      </c>
+      <c r="G19" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -843,15 +871,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DB002FF-49E8-4F00-BBA1-9E981B1CFB66}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="11.375" customWidth="1"/>
-    <col min="3" max="3" width="16.625" customWidth="1"/>
+    <col min="3" max="3" width="23.875" customWidth="1"/>
     <col min="4" max="4" width="17.375" customWidth="1"/>
+    <col min="5" max="5" width="13.875" customWidth="1"/>
+    <col min="6" max="6" width="24.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -862,10 +892,16 @@
         <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+      <c r="E1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>80</v>
       </c>
@@ -876,7 +912,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>80</v>
       </c>
@@ -887,7 +923,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>68</v>
       </c>
@@ -898,7 +934,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>82</v>
       </c>
@@ -909,7 +945,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>91</v>
       </c>
@@ -920,7 +956,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>99</v>
       </c>
@@ -931,7 +967,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>99</v>
       </c>
@@ -939,10 +975,10 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>101</v>
       </c>
@@ -950,10 +986,10 @@
         <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="D9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -963,7 +999,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA9FDAFF-FC45-49EA-B8F5-53ECA0B0E905}">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.25" customWidth="1"/>
@@ -1069,7 +1105,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
+      <c r="A12" t="s">
         <v>0</v>
       </c>
       <c r="B12" t="s">
@@ -1077,7 +1113,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
+      <c r="A13" t="s">
         <v>5</v>
       </c>
       <c r="B13" t="s">
@@ -1085,7 +1121,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B14" t="s">
@@ -1096,7 +1132,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="4"/>
+      <c r="A15" s="3"/>
       <c r="B15" t="s">
         <v>12</v>
       </c>
@@ -1105,18 +1141,18 @@
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="4"/>
+      <c r="A16" s="3"/>
       <c r="B16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C16" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="15" x14ac:dyDescent="0.25">
-      <c r="A17" s="4"/>
+      <c r="A17" s="3"/>
       <c r="B17" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="C17" t="s">
         <v>43</v>
@@ -1124,13 +1160,24 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B18" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C18" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
         <v>49</v>
+      </c>
+      <c r="B19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added a surveillance method to find missing/hidden properties in an area
</commit_message>
<xml_diff>
--- a/scenarios/v06/new_actions_1.xlsx
+++ b/scenarios/v06/new_actions_1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thaophuongl\Documents\HASTE_CODE\OutbreakSimulator\scenarios\v06\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFD1238B-2017-427C-886D-C62402C0405E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81FA8CC8-6638-48B0-8896-F26FD4703259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{01539856-3AD6-4856-AAFB-F25B45651A69}"/>
+    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{01539856-3AD6-4856-AAFB-F25B45651A69}"/>
   </bookViews>
   <sheets>
     <sheet name="jobs" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="79">
   <si>
     <t>ID</t>
   </si>
@@ -271,6 +271,12 @@
   </si>
   <si>
     <t>A parameter to adjust the increase of passive surveillance reports</t>
+  </si>
+  <si>
+    <t>Missing Properties Survey</t>
+  </si>
+  <si>
+    <t>uncovers any "missing" (i.e, unknown) properties in the area</t>
   </si>
 </sst>
 </file>
@@ -484,9 +490,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -508,47 +511,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -564,12 +528,54 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -580,9 +586,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1405,7 +1411,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1413,120 +1419,120 @@
       <c r="A2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="22"/>
-      <c r="D2" s="23"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="40"/>
       <c r="F2" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="G2" s="35" t="s">
+      <c r="G2" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="H2" s="36"/>
+      <c r="H2" s="22"/>
     </row>
     <row r="3" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="33"/>
-      <c r="D3" s="34"/>
-      <c r="F3" s="15" t="s">
+      <c r="C3" s="41"/>
+      <c r="D3" s="42"/>
+      <c r="F3" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="37" t="s">
+      <c r="G3" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="H3" s="38"/>
+      <c r="H3" s="24"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="33"/>
-      <c r="D4" s="34"/>
-      <c r="F4" s="15" t="s">
+      <c r="C4" s="41"/>
+      <c r="D4" s="42"/>
+      <c r="F4" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="39" t="s">
+      <c r="G4" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="H4" s="40"/>
+      <c r="H4" s="26"/>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="25"/>
-      <c r="D5" s="26"/>
-      <c r="F5" s="15" t="s">
+      <c r="C5" s="20"/>
+      <c r="D5" s="31"/>
+      <c r="F5" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="39" t="s">
+      <c r="G5" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="H5" s="40"/>
+      <c r="H5" s="26"/>
     </row>
     <row r="6" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="C6" s="25"/>
-      <c r="D6" s="26"/>
-      <c r="F6" s="15" t="s">
+      <c r="C6" s="20"/>
+      <c r="D6" s="31"/>
+      <c r="F6" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="37" t="s">
+      <c r="G6" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="H6" s="38"/>
+      <c r="H6" s="24"/>
     </row>
     <row r="7" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="C7" s="25"/>
-      <c r="D7" s="26"/>
-      <c r="F7" s="15" t="s">
+      <c r="C7" s="20"/>
+      <c r="D7" s="31"/>
+      <c r="F7" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="41" t="s">
+      <c r="G7" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="H7" s="42"/>
+      <c r="H7" s="36"/>
     </row>
     <row r="8" spans="1:8" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="33"/>
-      <c r="D8" s="34"/>
-      <c r="F8" s="16" t="s">
+      <c r="C8" s="41"/>
+      <c r="D8" s="42"/>
+      <c r="F8" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="G8" s="27" t="s">
+      <c r="G8" s="37" t="s">
         <v>70</v>
       </c>
-      <c r="H8" s="28"/>
+      <c r="H8" s="29"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
@@ -1544,25 +1550,25 @@
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="12" t="s">
+      <c r="E12" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="F12" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="G12" s="12" t="s">
+      <c r="G12" s="11" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1570,7 +1576,7 @@
       <c r="A13" s="4">
         <v>68</v>
       </c>
-      <c r="B13" s="13">
+      <c r="B13" s="12">
         <v>46034</v>
       </c>
       <c r="C13" s="4" t="s">
@@ -1579,7 +1585,7 @@
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
-      <c r="G13" s="14" t="s">
+      <c r="G13" s="13" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1587,7 +1593,7 @@
       <c r="A14" s="4">
         <v>68</v>
       </c>
-      <c r="B14" s="13">
+      <c r="B14" s="12">
         <v>46034</v>
       </c>
       <c r="C14" s="4" t="s">
@@ -1602,7 +1608,7 @@
       <c r="A15" s="4">
         <v>68</v>
       </c>
-      <c r="B15" s="13">
+      <c r="B15" s="12">
         <v>46034</v>
       </c>
       <c r="C15" s="4" t="s">
@@ -1619,7 +1625,7 @@
       <c r="A16" s="4">
         <v>80</v>
       </c>
-      <c r="B16" s="13">
+      <c r="B16" s="12">
         <v>46035</v>
       </c>
       <c r="C16" s="4" t="s">
@@ -1638,7 +1644,7 @@
       <c r="A17" s="4">
         <v>100</v>
       </c>
-      <c r="B17" s="13">
+      <c r="B17" s="12">
         <v>46036</v>
       </c>
       <c r="C17" s="4" t="s">
@@ -1657,7 +1663,7 @@
       <c r="A18" s="4">
         <v>101</v>
       </c>
-      <c r="B18" s="13">
+      <c r="B18" s="12">
         <v>46036</v>
       </c>
       <c r="C18" s="4" t="s">
@@ -1674,7 +1680,7 @@
       <c r="A19" s="4">
         <v>500</v>
       </c>
-      <c r="B19" s="13">
+      <c r="B19" s="12">
         <v>46036</v>
       </c>
       <c r="C19" s="4" t="s">
@@ -1697,7 +1703,7 @@
       <c r="E22" s="2"/>
     </row>
     <row r="23" spans="1:8" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A23" s="17" t="s">
+      <c r="A23" s="16" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1705,29 +1711,29 @@
       <c r="A24" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B24" s="21" t="s">
+      <c r="B24" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="C24" s="22"/>
-      <c r="D24" s="23"/>
+      <c r="C24" s="39"/>
+      <c r="D24" s="40"/>
       <c r="F24" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="G24" s="35" t="s">
+      <c r="G24" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="36"/>
+      <c r="H24" s="22"/>
     </row>
     <row r="25" spans="1:8" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="24" t="s">
+      <c r="B25" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="C25" s="25"/>
-      <c r="D25" s="26"/>
-      <c r="F25" s="18" t="s">
+      <c r="C25" s="20"/>
+      <c r="D25" s="31"/>
+      <c r="F25" s="17" t="s">
         <v>51</v>
       </c>
       <c r="G25" s="9" t="s">
@@ -1739,84 +1745,88 @@
       <c r="A26" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="24" t="s">
+      <c r="B26" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="C26" s="25"/>
-      <c r="D26" s="26"/>
-      <c r="F26" s="18" t="s">
+      <c r="C26" s="20"/>
+      <c r="D26" s="31"/>
+      <c r="F26" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="G26" s="46" t="s">
+      <c r="G26" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="H26" s="40"/>
+      <c r="H26" s="26"/>
     </row>
     <row r="27" spans="1:8" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B27" s="24" t="s">
+      <c r="B27" s="30" t="s">
         <v>59</v>
       </c>
-      <c r="C27" s="25"/>
-      <c r="D27" s="26"/>
-      <c r="F27" s="20" t="s">
+      <c r="C27" s="20"/>
+      <c r="D27" s="31"/>
+      <c r="F27" s="17" t="s">
         <v>72</v>
       </c>
       <c r="G27" s="47" t="s">
         <v>65</v>
       </c>
-      <c r="H27" s="28"/>
+      <c r="H27" s="24"/>
     </row>
     <row r="28" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="24" t="s">
+      <c r="B28" s="30" t="s">
         <v>73</v>
       </c>
-      <c r="C28" s="25"/>
-      <c r="D28" s="26"/>
-      <c r="F28" s="19"/>
-      <c r="G28" s="11"/>
-      <c r="H28" s="11"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="31"/>
+      <c r="F28" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="G28" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="H28" s="29"/>
     </row>
     <row r="29" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B29" s="24" t="s">
+      <c r="B29" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="C29" s="25"/>
-      <c r="D29" s="26"/>
-      <c r="F29" s="19"/>
-      <c r="G29" s="37"/>
-      <c r="H29" s="37"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="31"/>
+      <c r="F29" s="18"/>
+      <c r="G29" s="23"/>
+      <c r="H29" s="23"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B30" s="24" t="s">
+      <c r="B30" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="C30" s="25"/>
-      <c r="D30" s="26"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="31"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B31" s="29" t="s">
+      <c r="B31" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="C31" s="30"/>
-      <c r="D31" s="31"/>
+      <c r="C31" s="33"/>
+      <c r="D31" s="34"/>
     </row>
     <row r="33" spans="1:8" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A33" s="17" t="s">
+      <c r="A33" s="16" t="s">
         <v>69</v>
       </c>
     </row>
@@ -1824,101 +1834,101 @@
       <c r="A34" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B34" s="21" t="s">
+      <c r="B34" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="C34" s="22"/>
-      <c r="D34" s="23"/>
+      <c r="C34" s="39"/>
+      <c r="D34" s="40"/>
       <c r="F34" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="G34" s="35" t="s">
+      <c r="G34" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="H34" s="36"/>
+      <c r="H34" s="22"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B35" s="24" t="s">
+      <c r="B35" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="C35" s="25"/>
-      <c r="D35" s="26"/>
-      <c r="F35" s="15" t="s">
+      <c r="C35" s="20"/>
+      <c r="D35" s="31"/>
+      <c r="F35" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="G35" s="37" t="s">
+      <c r="G35" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="H35" s="38"/>
+      <c r="H35" s="24"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B36" s="24" t="s">
+      <c r="B36" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="C36" s="25"/>
-      <c r="D36" s="26"/>
-      <c r="F36" s="15" t="s">
+      <c r="C36" s="20"/>
+      <c r="D36" s="31"/>
+      <c r="F36" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="G36" s="39" t="s">
+      <c r="G36" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="H36" s="40"/>
+      <c r="H36" s="26"/>
     </row>
     <row r="37" spans="1:8" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>57</v>
       </c>
-      <c r="B37" s="24" t="s">
+      <c r="B37" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="C37" s="25"/>
-      <c r="D37" s="26"/>
-      <c r="F37" s="20" t="s">
+      <c r="C37" s="20"/>
+      <c r="D37" s="31"/>
+      <c r="F37" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="G37" s="27" t="s">
+      <c r="G37" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="H37" s="28"/>
+      <c r="H37" s="29"/>
     </row>
     <row r="38" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B38" s="24" t="s">
+      <c r="B38" s="30" t="s">
         <v>76</v>
       </c>
-      <c r="C38" s="25"/>
-      <c r="D38" s="26"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="31"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B39" s="29" t="s">
+      <c r="B39" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="C39" s="30"/>
-      <c r="D39" s="31"/>
+      <c r="C39" s="33"/>
+      <c r="D39" s="34"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A40" s="19"/>
-      <c r="B40" s="25"/>
-      <c r="C40" s="25"/>
-      <c r="D40" s="25"/>
+      <c r="A40" s="18"/>
+      <c r="B40" s="20"/>
+      <c r="C40" s="20"/>
+      <c r="D40" s="20"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A41" s="19"/>
-      <c r="B41" s="25"/>
-      <c r="C41" s="25"/>
-      <c r="D41" s="25"/>
+      <c r="A41" s="18"/>
+      <c r="B41" s="20"/>
+      <c r="C41" s="20"/>
+      <c r="D41" s="20"/>
     </row>
     <row r="42" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
@@ -1929,7 +1939,31 @@
       <c r="C43" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="39">
+  <mergeCells count="40">
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
     <mergeCell ref="B41:D41"/>
     <mergeCell ref="G34:H34"/>
     <mergeCell ref="G35:H35"/>
@@ -1943,32 +1977,9 @@
     <mergeCell ref="B38:D38"/>
     <mergeCell ref="B39:D39"/>
     <mergeCell ref="B40:D40"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B6:D6"/>
     <mergeCell ref="B34:D34"/>
     <mergeCell ref="B35:D35"/>
     <mergeCell ref="G37:H37"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="B31:D31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
initial set up of funciton to auto-generate jobs
</commit_message>
<xml_diff>
--- a/scenarios/v06/new_actions_1.xlsx
+++ b/scenarios/v06/new_actions_1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thaophuongl\Documents\HASTE_CODE\OutbreakSimulator\scenarios\v06\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81FA8CC8-6638-48B0-8896-F26FD4703259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B374AC7-AA15-450F-9173-B4F259974BAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{01539856-3AD6-4856-AAFB-F25B45651A69}"/>
+    <workbookView xWindow="-80" yWindow="-80" windowWidth="23200" windowHeight="14800" xr2:uid="{01539856-3AD6-4856-AAFB-F25B45651A69}"/>
   </bookViews>
   <sheets>
     <sheet name="jobs" sheetId="1" r:id="rId1"/>
@@ -468,7 +468,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -511,8 +511,47 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -528,68 +567,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1188,6 +1185,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1419,120 +1417,120 @@
       <c r="A2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="39"/>
-      <c r="D2" s="40"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="30"/>
       <c r="F2" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="34" t="s">
         <v>42</v>
       </c>
-      <c r="H2" s="22"/>
+      <c r="H2" s="35"/>
     </row>
     <row r="3" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="42"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="33"/>
       <c r="F3" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="23" t="s">
+      <c r="G3" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="H3" s="24"/>
+      <c r="H3" s="37"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="46" t="s">
+      <c r="B4" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="41"/>
-      <c r="D4" s="42"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="33"/>
       <c r="F4" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="25" t="s">
+      <c r="G4" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="H4" s="26"/>
+      <c r="H4" s="39"/>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="20"/>
-      <c r="D5" s="31"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="24"/>
       <c r="F5" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="25" t="s">
+      <c r="G5" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="H5" s="26"/>
+      <c r="H5" s="39"/>
     </row>
     <row r="6" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="C6" s="20"/>
-      <c r="D6" s="31"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="24"/>
       <c r="F6" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="23" t="s">
+      <c r="G6" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="H6" s="24"/>
+      <c r="H6" s="37"/>
     </row>
     <row r="7" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="30" t="s">
+      <c r="B7" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="C7" s="20"/>
-      <c r="D7" s="31"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="24"/>
       <c r="F7" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="35" t="s">
+      <c r="G7" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="H7" s="36"/>
+      <c r="H7" s="41"/>
     </row>
     <row r="8" spans="1:8" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="30" t="s">
+      <c r="B8" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="41"/>
-      <c r="D8" s="42"/>
+      <c r="C8" s="32"/>
+      <c r="D8" s="33"/>
       <c r="F8" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="G8" s="37" t="s">
+      <c r="G8" s="42" t="s">
         <v>70</v>
       </c>
-      <c r="H8" s="29"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
@@ -1711,28 +1709,28 @@
       <c r="A24" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B24" s="38" t="s">
+      <c r="B24" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="C24" s="39"/>
-      <c r="D24" s="40"/>
+      <c r="C24" s="29"/>
+      <c r="D24" s="30"/>
       <c r="F24" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="G24" s="21" t="s">
+      <c r="G24" s="34" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="22"/>
+      <c r="H24" s="35"/>
     </row>
     <row r="25" spans="1:8" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="30" t="s">
+      <c r="B25" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="C25" s="20"/>
-      <c r="D25" s="31"/>
+      <c r="C25" s="23"/>
+      <c r="D25" s="24"/>
       <c r="F25" s="17" t="s">
         <v>51</v>
       </c>
@@ -1745,85 +1743,85 @@
       <c r="A26" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="30" t="s">
+      <c r="B26" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="C26" s="20"/>
-      <c r="D26" s="31"/>
+      <c r="C26" s="23"/>
+      <c r="D26" s="24"/>
       <c r="F26" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="G26" s="27" t="s">
+      <c r="G26" s="46" t="s">
         <v>67</v>
       </c>
-      <c r="H26" s="26"/>
+      <c r="H26" s="39"/>
     </row>
     <row r="27" spans="1:8" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B27" s="30" t="s">
+      <c r="B27" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="C27" s="20"/>
-      <c r="D27" s="31"/>
+      <c r="C27" s="23"/>
+      <c r="D27" s="24"/>
       <c r="F27" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="G27" s="47" t="s">
+      <c r="G27" s="36" t="s">
         <v>65</v>
       </c>
-      <c r="H27" s="24"/>
+      <c r="H27" s="37"/>
     </row>
     <row r="28" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="30" t="s">
+      <c r="B28" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="C28" s="20"/>
-      <c r="D28" s="31"/>
+      <c r="C28" s="23"/>
+      <c r="D28" s="24"/>
       <c r="F28" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="G28" s="28" t="s">
+      <c r="G28" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="H28" s="29"/>
+      <c r="H28" s="21"/>
     </row>
     <row r="29" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B29" s="30" t="s">
+      <c r="B29" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="C29" s="20"/>
-      <c r="D29" s="31"/>
+      <c r="C29" s="23"/>
+      <c r="D29" s="24"/>
       <c r="F29" s="18"/>
-      <c r="G29" s="23"/>
-      <c r="H29" s="23"/>
+      <c r="G29" s="36"/>
+      <c r="H29" s="36"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B30" s="30" t="s">
+      <c r="B30" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="C30" s="20"/>
-      <c r="D30" s="31"/>
+      <c r="C30" s="23"/>
+      <c r="D30" s="24"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B31" s="32" t="s">
+      <c r="B31" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="C31" s="33"/>
-      <c r="D31" s="34"/>
+      <c r="C31" s="26"/>
+      <c r="D31" s="27"/>
     </row>
     <row r="33" spans="1:8" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A33" s="16" t="s">
@@ -1834,101 +1832,101 @@
       <c r="A34" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B34" s="38" t="s">
+      <c r="B34" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="C34" s="39"/>
-      <c r="D34" s="40"/>
+      <c r="C34" s="29"/>
+      <c r="D34" s="30"/>
       <c r="F34" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="G34" s="21" t="s">
+      <c r="G34" s="34" t="s">
         <v>62</v>
       </c>
-      <c r="H34" s="22"/>
+      <c r="H34" s="35"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B35" s="30" t="s">
+      <c r="B35" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="C35" s="20"/>
-      <c r="D35" s="31"/>
+      <c r="C35" s="23"/>
+      <c r="D35" s="24"/>
       <c r="F35" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="G35" s="23" t="s">
+      <c r="G35" s="36" t="s">
         <v>63</v>
       </c>
-      <c r="H35" s="24"/>
+      <c r="H35" s="37"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B36" s="30" t="s">
+      <c r="B36" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C36" s="20"/>
-      <c r="D36" s="31"/>
+      <c r="C36" s="23"/>
+      <c r="D36" s="24"/>
       <c r="F36" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="G36" s="25" t="s">
+      <c r="G36" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="H36" s="26"/>
+      <c r="H36" s="39"/>
     </row>
     <row r="37" spans="1:8" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>57</v>
       </c>
-      <c r="B37" s="30" t="s">
+      <c r="B37" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="C37" s="20"/>
-      <c r="D37" s="31"/>
+      <c r="C37" s="23"/>
+      <c r="D37" s="24"/>
       <c r="F37" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="G37" s="37" t="s">
+      <c r="G37" s="42" t="s">
         <v>68</v>
       </c>
-      <c r="H37" s="29"/>
+      <c r="H37" s="21"/>
     </row>
     <row r="38" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B38" s="30" t="s">
+      <c r="B38" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="C38" s="20"/>
-      <c r="D38" s="31"/>
+      <c r="C38" s="23"/>
+      <c r="D38" s="24"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B39" s="32" t="s">
+      <c r="B39" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="C39" s="33"/>
-      <c r="D39" s="34"/>
+      <c r="C39" s="26"/>
+      <c r="D39" s="27"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="18"/>
-      <c r="B40" s="20"/>
-      <c r="C40" s="20"/>
-      <c r="D40" s="20"/>
+      <c r="B40" s="23"/>
+      <c r="C40" s="23"/>
+      <c r="D40" s="23"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" s="18"/>
-      <c r="B41" s="20"/>
-      <c r="C41" s="20"/>
-      <c r="D41" s="20"/>
+      <c r="B41" s="23"/>
+      <c r="C41" s="23"/>
+      <c r="D41" s="23"/>
     </row>
     <row r="42" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
@@ -1940,30 +1938,6 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="G28:H28"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
     <mergeCell ref="B41:D41"/>
     <mergeCell ref="G34:H34"/>
     <mergeCell ref="G35:H35"/>
@@ -1980,6 +1954,30 @@
     <mergeCell ref="B34:D34"/>
     <mergeCell ref="B35:D35"/>
     <mergeCell ref="G37:H37"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B30:D30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>